<commit_message>
Extend parametrization review to multi-scenario with consistency sweep
- Z_AUX_apply_parametrization_review.py: process BAU (PWR+Tx) and INV (PWR only); add post-write consistency sweep enforcing per-year and cumulative max-capacity invariants via shared _xlsx_validation_core
- B1_Compiler.py: hook pre-solver validation (B1b_Pre_solver_validation) gated by pre_solver_validation config flag
- Config_MOMF_T1_AB.yaml: disable del_files, only_main_scenario and parallel for full multi-scenario debug runs
- Refresh A-Xtra_Emissions, A-Xtra_Storage, CapacityAndDistances and Secondary_Techs_Editor inputs
</commit_message>
<xml_diff>
--- a/t1_confection/CapacityAndDistances.xlsx
+++ b/t1_confection/CapacityAndDistances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\relac_tx\t1_confection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17AC5D30-6F52-4051-A2E9-2212DE461891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD2E1BD-D5D7-45BA-A42F-A1E84E9560AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0C96E5F6-F950-4B3A-9DA0-C225FFFF14E3}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0C96E5F6-F950-4B3A-9DA0-C225FFFF14E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="34">
   <si>
     <t>Country</t>
   </si>
@@ -135,6 +135,12 @@
   </si>
   <si>
     <t>NDC_SinInterconexiones</t>
+  </si>
+  <si>
+    <t>OPT</t>
+  </si>
+  <si>
+    <t>INV</t>
   </si>
 </sst>
 </file>
@@ -514,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F5565BA-9CF5-4FA5-B374-01C254CE755C}">
-  <dimension ref="A1:M157"/>
+  <dimension ref="A1:M191"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
@@ -3134,24 +3140,662 @@
       <c r="M153" s="1"/>
     </row>
     <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>32</v>
+      </c>
+      <c r="B154" t="s">
+        <v>4</v>
+      </c>
+      <c r="C154">
+        <v>6.3341098032793836E-2</v>
+      </c>
+      <c r="D154">
+        <v>88.22</v>
+      </c>
+      <c r="E154">
+        <v>38.049999999999997</v>
+      </c>
       <c r="K154" s="1"/>
       <c r="L154" s="1"/>
       <c r="M154" s="1"/>
     </row>
     <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>32</v>
+      </c>
+      <c r="B155" t="s">
+        <v>5</v>
+      </c>
+      <c r="C155">
+        <v>0.39438796888343336</v>
+      </c>
+      <c r="D155">
+        <v>186.34</v>
+      </c>
+      <c r="E155">
+        <v>85.73</v>
+      </c>
       <c r="K155" s="1"/>
       <c r="L155" s="1"/>
       <c r="M155" s="1"/>
     </row>
     <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>32</v>
+      </c>
+      <c r="B156" t="s">
+        <v>6</v>
+      </c>
+      <c r="C156">
+        <v>0.33913554812198615</v>
+      </c>
+      <c r="D156">
+        <v>256.02027210884359</v>
+      </c>
+      <c r="E156">
+        <v>192.17599999999999</v>
+      </c>
       <c r="K156" s="1"/>
       <c r="L156" s="1"/>
       <c r="M156" s="1"/>
     </row>
     <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>32</v>
+      </c>
+      <c r="B157" t="s">
+        <v>7</v>
+      </c>
+      <c r="C157">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D157">
+        <v>163.3391666666667</v>
+      </c>
+      <c r="E157">
+        <v>143.68</v>
+      </c>
       <c r="K157" s="1"/>
       <c r="L157" s="1"/>
       <c r="M157" s="1"/>
+    </row>
+    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>32</v>
+      </c>
+      <c r="B158" t="s">
+        <v>8</v>
+      </c>
+      <c r="C158">
+        <v>0.41430655317047549</v>
+      </c>
+      <c r="D158">
+        <v>108.5291304347826</v>
+      </c>
+      <c r="E158">
+        <v>98.22</v>
+      </c>
+    </row>
+    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>32</v>
+      </c>
+      <c r="B159" t="s">
+        <v>9</v>
+      </c>
+      <c r="C159">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D159">
+        <v>203.50200000000001</v>
+      </c>
+      <c r="E159">
+        <v>64.025000000000006</v>
+      </c>
+    </row>
+    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>32</v>
+      </c>
+      <c r="B160" t="s">
+        <v>10</v>
+      </c>
+      <c r="C160">
+        <v>0.41430655317047549</v>
+      </c>
+      <c r="D160">
+        <v>94.118333333333339</v>
+      </c>
+      <c r="E160">
+        <v>48.194999999999993</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>32</v>
+      </c>
+      <c r="B161" t="s">
+        <v>11</v>
+      </c>
+      <c r="C161">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D161">
+        <v>106.5366666666667</v>
+      </c>
+      <c r="E161">
+        <v>46.660833333333329</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>32</v>
+      </c>
+      <c r="B162" t="s">
+        <v>12</v>
+      </c>
+      <c r="C162">
+        <v>6.3341098032793836E-2</v>
+      </c>
+      <c r="D162">
+        <v>88.22</v>
+      </c>
+      <c r="E162">
+        <v>38.049999999999997</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>32</v>
+      </c>
+      <c r="B163" t="s">
+        <v>13</v>
+      </c>
+      <c r="C163">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D163">
+        <v>123.36279999999999</v>
+      </c>
+      <c r="E163">
+        <v>81.328000000000003</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>32</v>
+      </c>
+      <c r="B164" t="s">
+        <v>14</v>
+      </c>
+      <c r="C164">
+        <v>0.29081133059081449</v>
+      </c>
+      <c r="D164">
+        <v>122.0466666666667</v>
+      </c>
+      <c r="E164">
+        <v>48.417777777777779</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>32</v>
+      </c>
+      <c r="B165" t="s">
+        <v>15</v>
+      </c>
+      <c r="C165">
+        <v>0.46211115545937642</v>
+      </c>
+      <c r="D165">
+        <v>70.418750000000003</v>
+      </c>
+      <c r="E165">
+        <v>39.119999999999997</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>32</v>
+      </c>
+      <c r="B166" t="s">
+        <v>16</v>
+      </c>
+      <c r="C166">
+        <v>0.37724066588850141</v>
+      </c>
+      <c r="D166">
+        <v>131.62799999999999</v>
+      </c>
+      <c r="E166">
+        <v>131.62799999999999</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>32</v>
+      </c>
+      <c r="B167" t="s">
+        <v>17</v>
+      </c>
+      <c r="C167">
+        <v>0.33913554812198615</v>
+      </c>
+      <c r="D167">
+        <v>286.14368421052632</v>
+      </c>
+      <c r="E167">
+        <v>194.56100000000001</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>32</v>
+      </c>
+      <c r="B168" t="s">
+        <v>18</v>
+      </c>
+      <c r="C168">
+        <v>0.17448679835448869</v>
+      </c>
+      <c r="D168">
+        <v>88.22</v>
+      </c>
+      <c r="E168">
+        <v>38.049999999999997</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>32</v>
+      </c>
+      <c r="B169" t="s">
+        <v>19</v>
+      </c>
+      <c r="C169">
+        <v>0.17147302994931884</v>
+      </c>
+      <c r="D169">
+        <v>287.18985294117653</v>
+      </c>
+      <c r="E169">
+        <v>131.28</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>32</v>
+      </c>
+      <c r="B170" t="s">
+        <v>20</v>
+      </c>
+      <c r="C170">
+        <v>0.39438796888343336</v>
+      </c>
+      <c r="D170">
+        <v>393.02153374233131</v>
+      </c>
+      <c r="E170">
+        <v>352.42</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>32</v>
+      </c>
+      <c r="B171" t="s">
+        <v>21</v>
+      </c>
+      <c r="C171">
+        <v>0.85736514974659417</v>
+      </c>
+      <c r="D171">
+        <v>576.67268656716419</v>
+      </c>
+      <c r="E171">
+        <v>355.66</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>32</v>
+      </c>
+      <c r="B172" t="s">
+        <v>22</v>
+      </c>
+      <c r="C172">
+        <v>0.85736514974659417</v>
+      </c>
+      <c r="D172">
+        <v>628.98857142857139</v>
+      </c>
+      <c r="E172">
+        <v>365.81028571428573</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>33</v>
+      </c>
+      <c r="B173" t="s">
+        <v>4</v>
+      </c>
+      <c r="C173">
+        <v>6.3341098032793836E-2</v>
+      </c>
+      <c r="D173">
+        <v>88.22</v>
+      </c>
+      <c r="E173">
+        <v>38.049999999999997</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>33</v>
+      </c>
+      <c r="B174" t="s">
+        <v>5</v>
+      </c>
+      <c r="C174">
+        <v>0.39438796888343336</v>
+      </c>
+      <c r="D174">
+        <v>186.34</v>
+      </c>
+      <c r="E174">
+        <v>85.73</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>33</v>
+      </c>
+      <c r="B175" t="s">
+        <v>6</v>
+      </c>
+      <c r="C175">
+        <v>0.33913554812198615</v>
+      </c>
+      <c r="D175">
+        <v>256.02027210884359</v>
+      </c>
+      <c r="E175">
+        <v>192.17599999999999</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>33</v>
+      </c>
+      <c r="B176" t="s">
+        <v>7</v>
+      </c>
+      <c r="C176">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D176">
+        <v>163.3391666666667</v>
+      </c>
+      <c r="E176">
+        <v>143.68</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>33</v>
+      </c>
+      <c r="B177" t="s">
+        <v>8</v>
+      </c>
+      <c r="C177">
+        <v>0.41430655317047549</v>
+      </c>
+      <c r="D177">
+        <v>108.5291304347826</v>
+      </c>
+      <c r="E177">
+        <v>98.22</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>33</v>
+      </c>
+      <c r="B178" t="s">
+        <v>9</v>
+      </c>
+      <c r="C178">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D178">
+        <v>203.50200000000001</v>
+      </c>
+      <c r="E178">
+        <v>64.025000000000006</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>33</v>
+      </c>
+      <c r="B179" t="s">
+        <v>10</v>
+      </c>
+      <c r="C179">
+        <v>0.41430655317047549</v>
+      </c>
+      <c r="D179">
+        <v>94.118333333333339</v>
+      </c>
+      <c r="E179">
+        <v>48.194999999999993</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>33</v>
+      </c>
+      <c r="B180" t="s">
+        <v>11</v>
+      </c>
+      <c r="C180">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D180">
+        <v>106.5366666666667</v>
+      </c>
+      <c r="E180">
+        <v>46.660833333333329</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>33</v>
+      </c>
+      <c r="B181" t="s">
+        <v>12</v>
+      </c>
+      <c r="C181">
+        <v>6.3341098032793836E-2</v>
+      </c>
+      <c r="D181">
+        <v>88.22</v>
+      </c>
+      <c r="E181">
+        <v>38.049999999999997</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>33</v>
+      </c>
+      <c r="B182" t="s">
+        <v>13</v>
+      </c>
+      <c r="C182">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D182">
+        <v>123.36279999999999</v>
+      </c>
+      <c r="E182">
+        <v>81.328000000000003</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>33</v>
+      </c>
+      <c r="B183" t="s">
+        <v>14</v>
+      </c>
+      <c r="C183">
+        <v>0.29081133059081449</v>
+      </c>
+      <c r="D183">
+        <v>122.0466666666667</v>
+      </c>
+      <c r="E183">
+        <v>48.417777777777779</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>33</v>
+      </c>
+      <c r="B184" t="s">
+        <v>15</v>
+      </c>
+      <c r="C184">
+        <v>0.46211115545937642</v>
+      </c>
+      <c r="D184">
+        <v>70.418750000000003</v>
+      </c>
+      <c r="E184">
+        <v>39.119999999999997</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>33</v>
+      </c>
+      <c r="B185" t="s">
+        <v>16</v>
+      </c>
+      <c r="C185">
+        <v>0.37724066588850141</v>
+      </c>
+      <c r="D185">
+        <v>131.62799999999999</v>
+      </c>
+      <c r="E185">
+        <v>131.62799999999999</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>33</v>
+      </c>
+      <c r="B186" t="s">
+        <v>17</v>
+      </c>
+      <c r="C186">
+        <v>0.33913554812198615</v>
+      </c>
+      <c r="D186">
+        <v>286.14368421052632</v>
+      </c>
+      <c r="E186">
+        <v>194.56100000000001</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>33</v>
+      </c>
+      <c r="B187" t="s">
+        <v>18</v>
+      </c>
+      <c r="C187">
+        <v>0.17448679835448869</v>
+      </c>
+      <c r="D187">
+        <v>88.22</v>
+      </c>
+      <c r="E187">
+        <v>38.049999999999997</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>33</v>
+      </c>
+      <c r="B188" t="s">
+        <v>19</v>
+      </c>
+      <c r="C188">
+        <v>0.17147302994931884</v>
+      </c>
+      <c r="D188">
+        <v>287.18985294117653</v>
+      </c>
+      <c r="E188">
+        <v>131.28</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>33</v>
+      </c>
+      <c r="B189" t="s">
+        <v>20</v>
+      </c>
+      <c r="C189">
+        <v>0.39438796888343336</v>
+      </c>
+      <c r="D189">
+        <v>393.02153374233131</v>
+      </c>
+      <c r="E189">
+        <v>352.42</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>33</v>
+      </c>
+      <c r="B190" t="s">
+        <v>21</v>
+      </c>
+      <c r="C190">
+        <v>0.85736514974659417</v>
+      </c>
+      <c r="D190">
+        <v>576.67268656716419</v>
+      </c>
+      <c r="E190">
+        <v>355.66</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>33</v>
+      </c>
+      <c r="B191" t="s">
+        <v>22</v>
+      </c>
+      <c r="C191">
+        <v>0.85736514974659417</v>
+      </c>
+      <c r="D191">
+        <v>628.98857142857139</v>
+      </c>
+      <c r="E191">
+        <v>365.81028571428573</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E153" xr:uid="{4F5565BA-9CF5-4FA5-B374-01C254CE755C}"/>
@@ -3160,15 +3804,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101000F48F53D8446FB4EB61FD3AFE2640F25" ma:contentTypeVersion="10" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a214a3ba0c52ae00a3b9ea52e20da1dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7db9c71a-8f0f-4486-8c92-6242e053eab7" xmlns:ns3="8ae01698-3168-4e7f-b9e7-0ddc1c80de73" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1812e4edb338c892157ee4b16223776a" ns2:_="" ns3:_="">
     <xsd:import namespace="7db9c71a-8f0f-4486-8c92-6242e053eab7"/>
@@ -3357,6 +3992,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3369,14 +4013,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F224398-9CAE-4ABB-8BD0-D44A1FFE7284}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FDD807C-2497-4096-8FB6-8C801BBCCBC7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3391,6 +4027,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F224398-9CAE-4ABB-8BD0-D44A1FFE7284}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat(dashboard): escenario VGB + toggle eje X años/periodos + paleta teal; scripts auxiliares
Dashboard:
- dashboard_config.py / Z_AUX_generate_transmission_maps.py: añade el escenario
  VGB ("VEGETATIVO B") tras INV; alias INV->"VEGETATIVO A", VGB->"VEGETATIVO B";
  color violeta #b07aa1 por escenario.
- build_dashboard.py: alto del lienzo escala con el nº de escenarios; nuevo
  toggle de eje X (años vs periodos, con agregación promedio/suma); filtrado de
  series por leyenda con recálculo de la suma de referencia; paleta de UI teal
  (#00414D / #23978E / #DFE0E6).
- Figures/dashboard.html: regenerado.

Scripts auxiliares nuevos:
- D5_load_fuel_var_costs.py: carga VariableCost (USD/L -> M$/PJ) por escenario.
- Miscellaneous/preprocess_data_muio.py: preprocesado de datos MUIO/OSeMOSYS.
- _process_csv_for_dashboard.py: procesa Combined_Inputs_Outputs CSV al dashboard.

Datos:
- CapacityAndDistances.xlsx, Demanda CireLAC_GTER_WEO.xlsx, _dashboard_data.csv,
  cf_corregido_brasil.html.
</commit_message>
<xml_diff>
--- a/t1_confection/CapacityAndDistances.xlsx
+++ b/t1_confection/CapacityAndDistances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\relac_tx\t1_confection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD2E1BD-D5D7-45BA-A42F-A1E84E9560AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3BC0415-894D-46E4-A87C-B626C3A3076C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0C96E5F6-F950-4B3A-9DA0-C225FFFF14E3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0C96E5F6-F950-4B3A-9DA0-C225FFFF14E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="35">
   <si>
     <t>Country</t>
   </si>
@@ -141,6 +141,9 @@
   </si>
   <si>
     <t>INV</t>
+  </si>
+  <si>
+    <t>VGB</t>
   </si>
 </sst>
 </file>
@@ -520,16 +523,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F5565BA-9CF5-4FA5-B374-01C254CE755C}">
-  <dimension ref="A1:M191"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M210"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -546,7 +549,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -563,7 +566,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -580,7 +583,7 @@
         <v>85.73</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -597,7 +600,7 @@
         <v>192.17599999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -614,7 +617,7 @@
         <v>143.68</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -631,7 +634,7 @@
         <v>98.22</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -648,7 +651,7 @@
         <v>64.025000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -665,7 +668,7 @@
         <v>48.194999999999993</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -682,7 +685,7 @@
         <v>46.660833333333329</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -699,7 +702,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -716,7 +719,7 @@
         <v>81.328000000000003</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -733,7 +736,7 @@
         <v>48.417777777777779</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -750,7 +753,7 @@
         <v>39.119999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -767,7 +770,7 @@
         <v>131.62799999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -784,7 +787,7 @@
         <v>194.56100000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -801,7 +804,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -818,7 +821,7 @@
         <v>131.28</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -835,7 +838,7 @@
         <v>352.42</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -852,7 +855,7 @@
         <v>355.66</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -869,7 +872,7 @@
         <v>365.81028571428573</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -886,7 +889,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -903,7 +906,7 @@
         <v>85.73</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -920,7 +923,7 @@
         <v>192.17599999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -937,7 +940,7 @@
         <v>143.68</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -954,7 +957,7 @@
         <v>98.22</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -971,7 +974,7 @@
         <v>64.025000000000006</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -988,7 +991,7 @@
         <v>48.194999999999993</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>25</v>
       </c>
@@ -1005,7 +1008,7 @@
         <v>46.660833333333329</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>25</v>
       </c>
@@ -1022,7 +1025,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>25</v>
       </c>
@@ -1039,7 +1042,7 @@
         <v>81.328000000000003</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>25</v>
       </c>
@@ -1056,7 +1059,7 @@
         <v>48.417777777777779</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>25</v>
       </c>
@@ -1073,7 +1076,7 @@
         <v>39.119999999999997</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>25</v>
       </c>
@@ -1090,7 +1093,7 @@
         <v>131.62799999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>25</v>
       </c>
@@ -1107,7 +1110,7 @@
         <v>194.56100000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>25</v>
       </c>
@@ -1124,7 +1127,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>25</v>
       </c>
@@ -1141,7 +1144,7 @@
         <v>131.28</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>25</v>
       </c>
@@ -1158,7 +1161,7 @@
         <v>352.42</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>25</v>
       </c>
@@ -1175,7 +1178,7 @@
         <v>355.66</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>25</v>
       </c>
@@ -1192,7 +1195,7 @@
         <v>365.81028571428573</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>26</v>
       </c>
@@ -1209,7 +1212,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>26</v>
       </c>
@@ -1226,7 +1229,7 @@
         <v>85.73</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>26</v>
       </c>
@@ -1243,7 +1246,7 @@
         <v>192.17599999999999</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>26</v>
       </c>
@@ -1260,7 +1263,7 @@
         <v>143.68</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>26</v>
       </c>
@@ -1277,7 +1280,7 @@
         <v>98.22</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>26</v>
       </c>
@@ -1294,7 +1297,7 @@
         <v>64.025000000000006</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>26</v>
       </c>
@@ -1311,7 +1314,7 @@
         <v>48.194999999999993</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>26</v>
       </c>
@@ -1328,7 +1331,7 @@
         <v>46.660833333333329</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>26</v>
       </c>
@@ -1345,7 +1348,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>26</v>
       </c>
@@ -1362,7 +1365,7 @@
         <v>81.328000000000003</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>26</v>
       </c>
@@ -1379,7 +1382,7 @@
         <v>48.417777777777779</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>26</v>
       </c>
@@ -1396,7 +1399,7 @@
         <v>39.119999999999997</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>26</v>
       </c>
@@ -1413,7 +1416,7 @@
         <v>131.62799999999999</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>26</v>
       </c>
@@ -1430,7 +1433,7 @@
         <v>194.56100000000001</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>26</v>
       </c>
@@ -1447,7 +1450,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>26</v>
       </c>
@@ -1464,7 +1467,7 @@
         <v>131.28</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>26</v>
       </c>
@@ -1481,7 +1484,7 @@
         <v>352.42</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>26</v>
       </c>
@@ -1498,7 +1501,7 @@
         <v>355.66</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>26</v>
       </c>
@@ -1515,7 +1518,7 @@
         <v>365.81028571428573</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>27</v>
       </c>
@@ -1532,7 +1535,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>27</v>
       </c>
@@ -1549,7 +1552,7 @@
         <v>85.73</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>27</v>
       </c>
@@ -1566,7 +1569,7 @@
         <v>192.17599999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>27</v>
       </c>
@@ -1583,7 +1586,7 @@
         <v>143.68</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>27</v>
       </c>
@@ -1600,7 +1603,7 @@
         <v>98.22</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>27</v>
       </c>
@@ -1617,7 +1620,7 @@
         <v>64.025000000000006</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>27</v>
       </c>
@@ -1634,7 +1637,7 @@
         <v>48.194999999999993</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>27</v>
       </c>
@@ -1651,7 +1654,7 @@
         <v>46.660833333333329</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>27</v>
       </c>
@@ -1668,7 +1671,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>27</v>
       </c>
@@ -1685,7 +1688,7 @@
         <v>81.328000000000003</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>27</v>
       </c>
@@ -1702,7 +1705,7 @@
         <v>48.417777777777779</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>27</v>
       </c>
@@ -1719,7 +1722,7 @@
         <v>39.119999999999997</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>27</v>
       </c>
@@ -1736,7 +1739,7 @@
         <v>131.62799999999999</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>27</v>
       </c>
@@ -1753,7 +1756,7 @@
         <v>194.56100000000001</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>27</v>
       </c>
@@ -1770,7 +1773,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>27</v>
       </c>
@@ -1787,7 +1790,7 @@
         <v>131.28</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>27</v>
       </c>
@@ -1804,7 +1807,7 @@
         <v>352.42</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>27</v>
       </c>
@@ -1821,7 +1824,7 @@
         <v>355.66</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>27</v>
       </c>
@@ -1838,7 +1841,7 @@
         <v>365.81028571428573</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>28</v>
       </c>
@@ -1855,7 +1858,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>28</v>
       </c>
@@ -1872,7 +1875,7 @@
         <v>85.73</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>28</v>
       </c>
@@ -1889,7 +1892,7 @@
         <v>192.17599999999999</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>28</v>
       </c>
@@ -1906,7 +1909,7 @@
         <v>143.68</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>28</v>
       </c>
@@ -1923,7 +1926,7 @@
         <v>98.22</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>28</v>
       </c>
@@ -1940,7 +1943,7 @@
         <v>64.025000000000006</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>28</v>
       </c>
@@ -1957,7 +1960,7 @@
         <v>48.194999999999993</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>28</v>
       </c>
@@ -1974,7 +1977,7 @@
         <v>46.660833333333329</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>28</v>
       </c>
@@ -1991,7 +1994,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>28</v>
       </c>
@@ -2008,7 +2011,7 @@
         <v>81.328000000000003</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>28</v>
       </c>
@@ -2025,7 +2028,7 @@
         <v>48.417777777777779</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>28</v>
       </c>
@@ -2042,7 +2045,7 @@
         <v>39.119999999999997</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>28</v>
       </c>
@@ -2059,7 +2062,7 @@
         <v>131.62799999999999</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>28</v>
       </c>
@@ -2076,7 +2079,7 @@
         <v>194.56100000000001</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>28</v>
       </c>
@@ -2093,7 +2096,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>28</v>
       </c>
@@ -2110,7 +2113,7 @@
         <v>131.28</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>28</v>
       </c>
@@ -2127,7 +2130,7 @@
         <v>352.42</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>28</v>
       </c>
@@ -2144,7 +2147,7 @@
         <v>355.66</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>28</v>
       </c>
@@ -2161,7 +2164,7 @@
         <v>365.81028571428573</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>29</v>
       </c>
@@ -2178,7 +2181,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>29</v>
       </c>
@@ -2195,7 +2198,7 @@
         <v>85.73</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>29</v>
       </c>
@@ -2212,7 +2215,7 @@
         <v>192.17599999999999</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>29</v>
       </c>
@@ -2229,7 +2232,7 @@
         <v>143.68</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>29</v>
       </c>
@@ -2246,7 +2249,7 @@
         <v>98.22</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>29</v>
       </c>
@@ -2263,7 +2266,7 @@
         <v>64.025000000000006</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>29</v>
       </c>
@@ -2280,7 +2283,7 @@
         <v>48.194999999999993</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>29</v>
       </c>
@@ -2297,7 +2300,7 @@
         <v>46.660833333333329</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>29</v>
       </c>
@@ -2314,7 +2317,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>29</v>
       </c>
@@ -2331,7 +2334,7 @@
         <v>81.328000000000003</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>29</v>
       </c>
@@ -2348,7 +2351,7 @@
         <v>48.417777777777779</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>29</v>
       </c>
@@ -2365,7 +2368,7 @@
         <v>39.119999999999997</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>29</v>
       </c>
@@ -2382,7 +2385,7 @@
         <v>131.62799999999999</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>29</v>
       </c>
@@ -2399,7 +2402,7 @@
         <v>194.56100000000001</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>29</v>
       </c>
@@ -2416,7 +2419,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>29</v>
       </c>
@@ -2433,7 +2436,7 @@
         <v>131.28</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>29</v>
       </c>
@@ -2450,7 +2453,7 @@
         <v>352.42</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>29</v>
       </c>
@@ -2467,7 +2470,7 @@
         <v>355.66</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>29</v>
       </c>
@@ -2484,7 +2487,7 @@
         <v>365.81028571428573</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>30</v>
       </c>
@@ -2501,7 +2504,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>30</v>
       </c>
@@ -2518,7 +2521,7 @@
         <v>85.73</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>30</v>
       </c>
@@ -2535,7 +2538,7 @@
         <v>192.17599999999999</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>30</v>
       </c>
@@ -2552,7 +2555,7 @@
         <v>143.68</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>30</v>
       </c>
@@ -2569,7 +2572,7 @@
         <v>98.22</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>30</v>
       </c>
@@ -2586,7 +2589,7 @@
         <v>64.025000000000006</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>30</v>
       </c>
@@ -2603,7 +2606,7 @@
         <v>48.194999999999993</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>30</v>
       </c>
@@ -2620,7 +2623,7 @@
         <v>46.660833333333329</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>30</v>
       </c>
@@ -2637,7 +2640,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>30</v>
       </c>
@@ -2654,7 +2657,7 @@
         <v>81.328000000000003</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>30</v>
       </c>
@@ -2671,7 +2674,7 @@
         <v>48.417777777777779</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>30</v>
       </c>
@@ -2688,7 +2691,7 @@
         <v>39.119999999999997</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>30</v>
       </c>
@@ -2705,7 +2708,7 @@
         <v>131.62799999999999</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>30</v>
       </c>
@@ -2722,7 +2725,7 @@
         <v>194.56100000000001</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>30</v>
       </c>
@@ -2739,7 +2742,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>30</v>
       </c>
@@ -2756,7 +2759,7 @@
         <v>131.28</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>30</v>
       </c>
@@ -2773,7 +2776,7 @@
         <v>352.42</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>30</v>
       </c>
@@ -2790,7 +2793,7 @@
         <v>355.66</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>30</v>
       </c>
@@ -2807,7 +2810,7 @@
         <v>365.81028571428573</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>31</v>
       </c>
@@ -2824,7 +2827,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>31</v>
       </c>
@@ -2841,7 +2844,7 @@
         <v>85.73</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>31</v>
       </c>
@@ -2858,7 +2861,7 @@
         <v>192.17599999999999</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>31</v>
       </c>
@@ -2875,7 +2878,7 @@
         <v>143.68</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>31</v>
       </c>
@@ -2892,7 +2895,7 @@
         <v>98.22</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>31</v>
       </c>
@@ -2909,7 +2912,7 @@
         <v>64.025000000000006</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>31</v>
       </c>
@@ -2926,7 +2929,7 @@
         <v>48.194999999999993</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>31</v>
       </c>
@@ -2943,7 +2946,7 @@
         <v>46.660833333333329</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>31</v>
       </c>
@@ -2960,7 +2963,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>31</v>
       </c>
@@ -2977,7 +2980,7 @@
         <v>81.328000000000003</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>31</v>
       </c>
@@ -2994,7 +2997,7 @@
         <v>48.417777777777779</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>31</v>
       </c>
@@ -3011,7 +3014,7 @@
         <v>39.119999999999997</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>31</v>
       </c>
@@ -3028,7 +3031,7 @@
         <v>131.62799999999999</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>31</v>
       </c>
@@ -3045,7 +3048,7 @@
         <v>194.56100000000001</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>31</v>
       </c>
@@ -3062,7 +3065,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>31</v>
       </c>
@@ -3079,7 +3082,7 @@
         <v>131.28</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>31</v>
       </c>
@@ -3099,7 +3102,7 @@
       <c r="L151" s="1"/>
       <c r="M151" s="1"/>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>31</v>
       </c>
@@ -3119,7 +3122,7 @@
       <c r="L152" s="1"/>
       <c r="M152" s="1"/>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>31</v>
       </c>
@@ -3139,7 +3142,7 @@
       <c r="L153" s="1"/>
       <c r="M153" s="1"/>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>32</v>
       </c>
@@ -3159,7 +3162,7 @@
       <c r="L154" s="1"/>
       <c r="M154" s="1"/>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>32</v>
       </c>
@@ -3179,7 +3182,7 @@
       <c r="L155" s="1"/>
       <c r="M155" s="1"/>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>32</v>
       </c>
@@ -3199,7 +3202,7 @@
       <c r="L156" s="1"/>
       <c r="M156" s="1"/>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>32</v>
       </c>
@@ -3219,7 +3222,7 @@
       <c r="L157" s="1"/>
       <c r="M157" s="1"/>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>32</v>
       </c>
@@ -3236,7 +3239,7 @@
         <v>98.22</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>32</v>
       </c>
@@ -3253,7 +3256,7 @@
         <v>64.025000000000006</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>32</v>
       </c>
@@ -3270,7 +3273,7 @@
         <v>48.194999999999993</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>32</v>
       </c>
@@ -3287,7 +3290,7 @@
         <v>46.660833333333329</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>32</v>
       </c>
@@ -3304,7 +3307,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>32</v>
       </c>
@@ -3321,7 +3324,7 @@
         <v>81.328000000000003</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>32</v>
       </c>
@@ -3338,7 +3341,7 @@
         <v>48.417777777777779</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>32</v>
       </c>
@@ -3355,7 +3358,7 @@
         <v>39.119999999999997</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>32</v>
       </c>
@@ -3372,7 +3375,7 @@
         <v>131.62799999999999</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>32</v>
       </c>
@@ -3389,7 +3392,7 @@
         <v>194.56100000000001</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>32</v>
       </c>
@@ -3406,7 +3409,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>32</v>
       </c>
@@ -3423,7 +3426,7 @@
         <v>131.28</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>32</v>
       </c>
@@ -3440,7 +3443,7 @@
         <v>352.42</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>32</v>
       </c>
@@ -3457,7 +3460,7 @@
         <v>355.66</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>32</v>
       </c>
@@ -3474,7 +3477,7 @@
         <v>365.81028571428573</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>33</v>
       </c>
@@ -3491,7 +3494,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>33</v>
       </c>
@@ -3508,7 +3511,7 @@
         <v>85.73</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>33</v>
       </c>
@@ -3525,7 +3528,7 @@
         <v>192.17599999999999</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>33</v>
       </c>
@@ -3542,7 +3545,7 @@
         <v>143.68</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>33</v>
       </c>
@@ -3559,7 +3562,7 @@
         <v>98.22</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>33</v>
       </c>
@@ -3576,7 +3579,7 @@
         <v>64.025000000000006</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>33</v>
       </c>
@@ -3593,7 +3596,7 @@
         <v>48.194999999999993</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>33</v>
       </c>
@@ -3610,7 +3613,7 @@
         <v>46.660833333333329</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>33</v>
       </c>
@@ -3627,7 +3630,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>33</v>
       </c>
@@ -3644,7 +3647,7 @@
         <v>81.328000000000003</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>33</v>
       </c>
@@ -3661,7 +3664,7 @@
         <v>48.417777777777779</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>33</v>
       </c>
@@ -3678,7 +3681,7 @@
         <v>39.119999999999997</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>33</v>
       </c>
@@ -3695,7 +3698,7 @@
         <v>131.62799999999999</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>33</v>
       </c>
@@ -3712,7 +3715,7 @@
         <v>194.56100000000001</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>33</v>
       </c>
@@ -3729,7 +3732,7 @@
         <v>38.049999999999997</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>33</v>
       </c>
@@ -3746,7 +3749,7 @@
         <v>131.28</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>33</v>
       </c>
@@ -3763,7 +3766,7 @@
         <v>352.42</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>33</v>
       </c>
@@ -3780,7 +3783,7 @@
         <v>355.66</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>33</v>
       </c>
@@ -3794,6 +3797,329 @@
         <v>628.98857142857139</v>
       </c>
       <c r="E191">
+        <v>365.81028571428573</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>34</v>
+      </c>
+      <c r="B192" t="s">
+        <v>4</v>
+      </c>
+      <c r="C192">
+        <v>6.3341098032793836E-2</v>
+      </c>
+      <c r="D192">
+        <v>88.22</v>
+      </c>
+      <c r="E192">
+        <v>38.049999999999997</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A193" t="s">
+        <v>34</v>
+      </c>
+      <c r="B193" t="s">
+        <v>5</v>
+      </c>
+      <c r="C193">
+        <v>0.39438796888343336</v>
+      </c>
+      <c r="D193">
+        <v>186.34</v>
+      </c>
+      <c r="E193">
+        <v>85.73</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A194" t="s">
+        <v>34</v>
+      </c>
+      <c r="B194" t="s">
+        <v>6</v>
+      </c>
+      <c r="C194">
+        <v>0.33913554812198615</v>
+      </c>
+      <c r="D194">
+        <v>256.02027210884359</v>
+      </c>
+      <c r="E194">
+        <v>192.17599999999999</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A195" t="s">
+        <v>34</v>
+      </c>
+      <c r="B195" t="s">
+        <v>7</v>
+      </c>
+      <c r="C195">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D195">
+        <v>163.3391666666667</v>
+      </c>
+      <c r="E195">
+        <v>143.68</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A196" t="s">
+        <v>34</v>
+      </c>
+      <c r="B196" t="s">
+        <v>8</v>
+      </c>
+      <c r="C196">
+        <v>0.41430655317047549</v>
+      </c>
+      <c r="D196">
+        <v>108.5291304347826</v>
+      </c>
+      <c r="E196">
+        <v>98.22</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A197" t="s">
+        <v>34</v>
+      </c>
+      <c r="B197" t="s">
+        <v>9</v>
+      </c>
+      <c r="C197">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D197">
+        <v>203.50200000000001</v>
+      </c>
+      <c r="E197">
+        <v>64.025000000000006</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A198" t="s">
+        <v>34</v>
+      </c>
+      <c r="B198" t="s">
+        <v>10</v>
+      </c>
+      <c r="C198">
+        <v>0.41430655317047549</v>
+      </c>
+      <c r="D198">
+        <v>94.118333333333339</v>
+      </c>
+      <c r="E198">
+        <v>48.194999999999993</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A199" t="s">
+        <v>34</v>
+      </c>
+      <c r="B199" t="s">
+        <v>11</v>
+      </c>
+      <c r="C199">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D199">
+        <v>106.5366666666667</v>
+      </c>
+      <c r="E199">
+        <v>46.660833333333329</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
+        <v>34</v>
+      </c>
+      <c r="B200" t="s">
+        <v>12</v>
+      </c>
+      <c r="C200">
+        <v>6.3341098032793836E-2</v>
+      </c>
+      <c r="D200">
+        <v>88.22</v>
+      </c>
+      <c r="E200">
+        <v>38.049999999999997</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
+        <v>34</v>
+      </c>
+      <c r="B201" t="s">
+        <v>13</v>
+      </c>
+      <c r="C201">
+        <v>0.35455080030934921</v>
+      </c>
+      <c r="D201">
+        <v>123.36279999999999</v>
+      </c>
+      <c r="E201">
+        <v>81.328000000000003</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A202" t="s">
+        <v>34</v>
+      </c>
+      <c r="B202" t="s">
+        <v>14</v>
+      </c>
+      <c r="C202">
+        <v>0.29081133059081449</v>
+      </c>
+      <c r="D202">
+        <v>122.0466666666667</v>
+      </c>
+      <c r="E202">
+        <v>48.417777777777779</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A203" t="s">
+        <v>34</v>
+      </c>
+      <c r="B203" t="s">
+        <v>15</v>
+      </c>
+      <c r="C203">
+        <v>0.46211115545937642</v>
+      </c>
+      <c r="D203">
+        <v>70.418750000000003</v>
+      </c>
+      <c r="E203">
+        <v>39.119999999999997</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A204" t="s">
+        <v>34</v>
+      </c>
+      <c r="B204" t="s">
+        <v>16</v>
+      </c>
+      <c r="C204">
+        <v>0.37724066588850141</v>
+      </c>
+      <c r="D204">
+        <v>131.62799999999999</v>
+      </c>
+      <c r="E204">
+        <v>131.62799999999999</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A205" t="s">
+        <v>34</v>
+      </c>
+      <c r="B205" t="s">
+        <v>17</v>
+      </c>
+      <c r="C205">
+        <v>0.33913554812198615</v>
+      </c>
+      <c r="D205">
+        <v>286.14368421052632</v>
+      </c>
+      <c r="E205">
+        <v>194.56100000000001</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A206" t="s">
+        <v>34</v>
+      </c>
+      <c r="B206" t="s">
+        <v>18</v>
+      </c>
+      <c r="C206">
+        <v>0.17448679835448869</v>
+      </c>
+      <c r="D206">
+        <v>88.22</v>
+      </c>
+      <c r="E206">
+        <v>38.049999999999997</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A207" t="s">
+        <v>34</v>
+      </c>
+      <c r="B207" t="s">
+        <v>19</v>
+      </c>
+      <c r="C207">
+        <v>0.17147302994931884</v>
+      </c>
+      <c r="D207">
+        <v>287.18985294117653</v>
+      </c>
+      <c r="E207">
+        <v>131.28</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A208" t="s">
+        <v>34</v>
+      </c>
+      <c r="B208" t="s">
+        <v>20</v>
+      </c>
+      <c r="C208">
+        <v>0.39438796888343336</v>
+      </c>
+      <c r="D208">
+        <v>393.02153374233131</v>
+      </c>
+      <c r="E208">
+        <v>352.42</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A209" t="s">
+        <v>34</v>
+      </c>
+      <c r="B209" t="s">
+        <v>21</v>
+      </c>
+      <c r="C209">
+        <v>0.85736514974659417</v>
+      </c>
+      <c r="D209">
+        <v>576.67268656716419</v>
+      </c>
+      <c r="E209">
+        <v>355.66</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A210" t="s">
+        <v>34</v>
+      </c>
+      <c r="B210" t="s">
+        <v>22</v>
+      </c>
+      <c r="C210">
+        <v>0.85736514974659417</v>
+      </c>
+      <c r="D210">
+        <v>628.98857142857139</v>
+      </c>
+      <c r="E210">
         <v>365.81028571428573</v>
       </c>
     </row>
@@ -3804,6 +4130,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101000F48F53D8446FB4EB61FD3AFE2640F25" ma:contentTypeVersion="10" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a214a3ba0c52ae00a3b9ea52e20da1dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7db9c71a-8f0f-4486-8c92-6242e053eab7" xmlns:ns3="8ae01698-3168-4e7f-b9e7-0ddc1c80de73" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1812e4edb338c892157ee4b16223776a" ns2:_="" ns3:_="">
     <xsd:import namespace="7db9c71a-8f0f-4486-8c92-6242e053eab7"/>
@@ -3992,15 +4327,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -4013,6 +4339,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F224398-9CAE-4ABB-8BD0-D44A1FFE7284}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FDD807C-2497-4096-8FB6-8C801BBCCBC7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4027,14 +4361,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F224398-9CAE-4ABB-8BD0-D44A1FFE7284}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>